<commit_message>
xlsx: embed all 45 training_dynamics PNGs directly in cells (visible without clicking links)
</commit_message>
<xml_diff>
--- a/on-the-fly-supervision.xlsx
+++ b/on-the-fly-supervision.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -28,9 +30,11 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <color rgb="000563C1"/>
+      <sz val="10"/>
       <u val="single"/>
     </font>
   </fonts>
@@ -73,16 +77,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -158,6 +165,1136 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>25</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>25</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>25</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2619375" cy="1619250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>25</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2619375" cy="1619250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2619375" cy="1619250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>25</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>25</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>25</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId22"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>25</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId23"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId24"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>25</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId26"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="27" name="Image 27" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId27"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId28"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>25</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId29"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId30"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId31"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>25</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId32"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId33"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId34"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>25</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId35"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId36"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId37"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>25</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId38"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId39"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId40"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>25</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId41"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId42"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId43"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>25</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId44"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2667000" cy="1581150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId45"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -452,12 +1589,12 @@
   <dimension ref="A1:AA16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
@@ -470,15 +1607,15 @@
     <col width="11" customWidth="1" min="16" max="16"/>
     <col width="11" customWidth="1" min="17" max="17"/>
     <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
     <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="30" customWidth="1" min="22" max="22"/>
+    <col width="26" customWidth="1" min="22" max="22"/>
     <col width="11" customWidth="1" min="23" max="23"/>
     <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="10" customWidth="1" min="25" max="25"/>
-    <col width="10" customWidth="1" min="26" max="26"/>
-    <col width="10" customWidth="1" min="27" max="27"/>
+    <col width="40" customWidth="1" min="25" max="25"/>
+    <col width="40" customWidth="1" min="26" max="26"/>
+    <col width="40" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -618,7 +1755,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
+    <row r="2" ht="135" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>baseline</t>
@@ -644,52 +1781,52 @@
           <t>full GT</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="4" t="n">
         <v>55986</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G2" s="4" t="n">
         <v>0.5972</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="4" t="n">
         <v>0.927</v>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="I2" s="4" t="n">
         <v>0.8287</v>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="J2" s="4" t="n">
         <v>0.442</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="K2" s="4" t="n">
         <v>0.6691</v>
       </c>
-      <c r="L2" s="2" t="n">
+      <c r="L2" s="4" t="n">
         <v>0.9323</v>
       </c>
-      <c r="M2" s="2" t="n">
+      <c r="M2" s="4" t="n">
         <v>0.8678</v>
       </c>
-      <c r="N2" s="2" t="n">
+      <c r="N2" s="4" t="n">
         <v>0.5395</v>
       </c>
-      <c r="O2" s="2" t="n">
+      <c r="O2" s="4" t="n">
         <v>0.7148</v>
       </c>
-      <c r="P2" s="2" t="n">
+      <c r="P2" s="4" t="n">
         <v>0.9335</v>
       </c>
-      <c r="Q2" s="2" t="n">
+      <c r="Q2" s="4" t="n">
         <v>0.8833</v>
       </c>
-      <c r="R2" s="2" t="n">
+      <c r="R2" s="4" t="n">
         <v>0.6057</v>
       </c>
-      <c r="S2" s="2" t="n">
+      <c r="S2" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="T2" s="2" t="n">
+      <c r="T2" s="4" t="n">
         <v>0.6959</v>
       </c>
-      <c r="U2" s="2" t="n">
+      <c r="U2" s="4" t="n">
         <v>0.5908</v>
       </c>
       <c r="V2" s="2" t="inlineStr">
@@ -697,29 +1834,14 @@
           <t>reference</t>
         </is>
       </c>
-      <c r="W2" s="2" t="n">
+      <c r="W2" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="X2" s="2" t="n">
+      <c r="X2" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="Y2" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="Z2" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="AA2" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
+    <row r="3" ht="135" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>v2 (cap=∞, no filter)</t>
@@ -745,52 +1867,52 @@
           <t>(1, 1, 0)</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="4" t="n">
         <v>49476</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="4" t="n">
         <v>0.6165</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="4" t="n">
         <v>0.9351</v>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="I3" s="4" t="n">
         <v>0.8473000000000001</v>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="4" t="n">
         <v>0.4636</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="K3" s="4" t="n">
         <v>0.6811</v>
       </c>
-      <c r="L3" s="2" t="n">
+      <c r="L3" s="4" t="n">
         <v>0.9393</v>
       </c>
-      <c r="M3" s="2" t="n">
+      <c r="M3" s="4" t="n">
         <v>0.8829</v>
       </c>
-      <c r="N3" s="2" t="n">
+      <c r="N3" s="4" t="n">
         <v>0.5512</v>
       </c>
-      <c r="O3" s="2" t="n">
+      <c r="O3" s="4" t="n">
         <v>0.7193000000000001</v>
       </c>
-      <c r="P3" s="2" t="n">
+      <c r="P3" s="4" t="n">
         <v>0.9401</v>
       </c>
-      <c r="Q3" s="2" t="n">
+      <c r="Q3" s="4" t="n">
         <v>0.8972</v>
       </c>
-      <c r="R3" s="2" t="n">
+      <c r="R3" s="4" t="n">
         <v>0.606</v>
       </c>
-      <c r="S3" s="2" t="n">
+      <c r="S3" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="T3" s="2" t="n">
+      <c r="T3" s="4" t="n">
         <v>0.6278</v>
       </c>
-      <c r="U3" s="2" t="n">
+      <c r="U3" s="4" t="n">
         <v>0.5065</v>
       </c>
       <c r="V3" s="2" t="inlineStr">
@@ -798,29 +1920,14 @@
           <t>2-seed; seed1 not in this row</t>
         </is>
       </c>
-      <c r="W3" s="2" t="n">
+      <c r="W3" s="4" t="n">
         <v>0.45</v>
       </c>
-      <c r="X3" s="2" t="n">
+      <c r="X3" s="4" t="n">
         <v>0.03</v>
       </c>
-      <c r="Y3" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="Z3" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="AA3" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
     </row>
-    <row r="4" ht="22" customHeight="1">
+    <row r="4" ht="135" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>c20 (cap=20, no filter)</t>
@@ -836,7 +1943,7 @@
           <t>pred==gt</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="4" t="n">
         <v>20</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -844,78 +1951,63 @@
           <t>(1, 1, 0)</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="4" t="n">
         <v>0.5929</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="4" t="n">
         <v>0.9262</v>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="I4" s="4" t="n">
         <v>0.8194</v>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="J4" s="4" t="n">
         <v>0.4391</v>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="K4" s="4" t="n">
         <v>0.6525</v>
       </c>
-      <c r="L4" s="2" t="n">
+      <c r="L4" s="4" t="n">
         <v>0.9318</v>
       </c>
-      <c r="M4" s="2" t="n">
+      <c r="M4" s="4" t="n">
         <v>0.8589</v>
       </c>
-      <c r="N4" s="2" t="n">
+      <c r="N4" s="4" t="n">
         <v>0.5168</v>
       </c>
-      <c r="O4" s="2" t="n">
+      <c r="O4" s="4" t="n">
         <v>0.6861</v>
       </c>
-      <c r="P4" s="2" t="n">
+      <c r="P4" s="4" t="n">
         <v>0.9332</v>
       </c>
-      <c r="Q4" s="2" t="n">
+      <c r="Q4" s="4" t="n">
         <v>0.8761</v>
       </c>
-      <c r="R4" s="2" t="n">
+      <c r="R4" s="4" t="n">
         <v>0.5629999999999999</v>
       </c>
-      <c r="S4" s="2" t="n">
+      <c r="S4" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="T4" s="2" t="n">
+      <c r="T4" s="4" t="n">
         <v>0.6861</v>
       </c>
-      <c r="U4" s="2" t="n">
+      <c r="U4" s="4" t="n">
         <v>0.5629999999999999</v>
       </c>
       <c r="V4" s="2" t="inlineStr"/>
-      <c r="W4" s="2" t="n">
+      <c r="W4" s="4" t="n">
         <v>-2.87</v>
       </c>
-      <c r="X4" s="2" t="n">
+      <c r="X4" s="4" t="n">
         <v>-4.27</v>
       </c>
-      <c r="Y4" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="Z4" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="AA4" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
+    <row r="5" ht="135" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>M3 (cap=10, no filter)</t>
@@ -931,7 +2023,7 @@
           <t>pred==gt</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="4" t="n">
         <v>10</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -939,78 +2031,63 @@
           <t>(1, 1, 0)</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="4" t="n">
         <v>63798</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G5" s="4" t="n">
         <v>0.5758</v>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="4" t="n">
         <v>0.9406</v>
       </c>
-      <c r="I5" s="2" t="n">
+      <c r="I5" s="4" t="n">
         <v>0.8233</v>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="J5" s="4" t="n">
         <v>0.4076</v>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="4" t="n">
         <v>0.6316000000000001</v>
       </c>
-      <c r="L5" s="2" t="n">
+      <c r="L5" s="4" t="n">
         <v>0.9448</v>
       </c>
-      <c r="M5" s="2" t="n">
+      <c r="M5" s="4" t="n">
         <v>0.8622</v>
       </c>
-      <c r="N5" s="2" t="n">
+      <c r="N5" s="4" t="n">
         <v>0.4799</v>
       </c>
-      <c r="O5" s="2" t="n">
+      <c r="O5" s="4" t="n">
         <v>0.664</v>
       </c>
-      <c r="P5" s="2" t="n">
+      <c r="P5" s="4" t="n">
         <v>0.9463</v>
       </c>
-      <c r="Q5" s="2" t="n">
+      <c r="Q5" s="4" t="n">
         <v>0.8768</v>
       </c>
-      <c r="R5" s="2" t="n">
+      <c r="R5" s="4" t="n">
         <v>0.5252</v>
       </c>
-      <c r="S5" s="2" t="n">
+      <c r="S5" s="4" t="n">
         <v>63798</v>
       </c>
-      <c r="T5" s="2" t="n">
+      <c r="T5" s="4" t="n">
         <v>0.664</v>
       </c>
-      <c r="U5" s="2" t="n">
+      <c r="U5" s="4" t="n">
         <v>0.5252</v>
       </c>
       <c r="V5" s="2" t="inlineStr"/>
-      <c r="W5" s="2" t="n">
+      <c r="W5" s="4" t="n">
         <v>-5.08</v>
       </c>
-      <c r="X5" s="2" t="n">
+      <c r="X5" s="4" t="n">
         <v>-8.050000000000001</v>
       </c>
-      <c r="Y5" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="Z5" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="AA5" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
     </row>
-    <row r="6" ht="22" customHeight="1">
+    <row r="6" ht="135" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>c5 (cap=5, no filter)</t>
@@ -1026,7 +2103,7 @@
           <t>pred==gt</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="4" t="n">
         <v>5</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1034,78 +2111,63 @@
           <t>(1, 1, 0)</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G6" s="4" t="n">
         <v>0.3382</v>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="4" t="n">
         <v>0.8374</v>
       </c>
-      <c r="I6" s="2" t="n">
+      <c r="I6" s="4" t="n">
         <v>0.4825</v>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="4" t="n">
         <v>0.1878</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="K6" s="4" t="n">
         <v>0.4005</v>
       </c>
-      <c r="L6" s="2" t="n">
+      <c r="L6" s="4" t="n">
         <v>0.8669</v>
       </c>
-      <c r="M6" s="2" t="n">
+      <c r="M6" s="4" t="n">
         <v>0.5619</v>
       </c>
-      <c r="N6" s="2" t="n">
+      <c r="N6" s="4" t="n">
         <v>0.2491</v>
       </c>
-      <c r="O6" s="2" t="n">
+      <c r="O6" s="4" t="n">
         <v>0.4404</v>
       </c>
-      <c r="P6" s="2" t="n">
+      <c r="P6" s="4" t="n">
         <v>0.8788</v>
       </c>
-      <c r="Q6" s="2" t="n">
+      <c r="Q6" s="4" t="n">
         <v>0.61</v>
       </c>
-      <c r="R6" s="2" t="n">
+      <c r="R6" s="4" t="n">
         <v>0.2907</v>
       </c>
-      <c r="S6" s="2" t="n">
+      <c r="S6" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="T6" s="2" t="n">
+      <c r="T6" s="4" t="n">
         <v>0.4404</v>
       </c>
-      <c r="U6" s="2" t="n">
+      <c r="U6" s="4" t="n">
         <v>0.2907</v>
       </c>
       <c r="V6" s="2" t="inlineStr"/>
-      <c r="W6" s="2" t="n">
+      <c r="W6" s="4" t="n">
         <v>-27.44</v>
       </c>
-      <c r="X6" s="2" t="n">
+      <c r="X6" s="4" t="n">
         <v>-31.5</v>
       </c>
-      <c r="Y6" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="Z6" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="AA6" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
+    <row r="7" ht="135" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>M2 (clue only)</t>
@@ -1131,78 +2193,63 @@
           <t>(1, 1, 0)</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G7" s="4" t="n">
         <v>0.2303</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="4" t="n">
         <v>0.8793</v>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="I7" s="4" t="n">
         <v>0.3335</v>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="4" t="n">
         <v>0.0693</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="K7" s="4" t="n">
         <v>0.2489</v>
       </c>
-      <c r="L7" s="2" t="n">
+      <c r="L7" s="4" t="n">
         <v>0.8957000000000001</v>
       </c>
-      <c r="M7" s="2" t="n">
+      <c r="M7" s="4" t="n">
         <v>0.3621</v>
       </c>
-      <c r="N7" s="2" t="n">
+      <c r="N7" s="4" t="n">
         <v>0.08409999999999999</v>
       </c>
-      <c r="O7" s="2" t="n">
+      <c r="O7" s="4" t="n">
         <v>0.2582</v>
       </c>
-      <c r="P7" s="2" t="n">
+      <c r="P7" s="4" t="n">
         <v>0.901</v>
       </c>
-      <c r="Q7" s="2" t="n">
+      <c r="Q7" s="4" t="n">
         <v>0.3757</v>
       </c>
-      <c r="R7" s="2" t="n">
+      <c r="R7" s="4" t="n">
         <v>0.0924</v>
       </c>
-      <c r="S7" s="2" t="n">
+      <c r="S7" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="T7" s="2" t="n">
+      <c r="T7" s="4" t="n">
         <v>0.2582</v>
       </c>
-      <c r="U7" s="2" t="n">
+      <c r="U7" s="4" t="n">
         <v>0.0924</v>
       </c>
       <c r="V7" s="2" t="inlineStr"/>
-      <c r="W7" s="2" t="n">
+      <c r="W7" s="4" t="n">
         <v>-45.66</v>
       </c>
-      <c r="X7" s="2" t="n">
+      <c r="X7" s="4" t="n">
         <v>-51.33</v>
       </c>
-      <c r="Y7" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="Z7" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="AA7" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
+    <row r="8" ht="135" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>inverse_mask cap=10</t>
@@ -1218,7 +2265,7 @@
           <t>pred==gt</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="4" t="n">
         <v>10</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1226,52 +2273,52 @@
           <t>(0.1, 0.1, 1.0)</t>
         </is>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="4" t="n">
         <v>62496</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G8" s="4" t="n">
         <v>0.5379</v>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="4" t="n">
         <v>0.9063</v>
       </c>
-      <c r="I8" s="2" t="n">
+      <c r="I8" s="4" t="n">
         <v>0.7974</v>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="J8" s="4" t="n">
         <v>0.3642</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="K8" s="4" t="n">
         <v>0.6071</v>
       </c>
-      <c r="L8" s="2" t="n">
+      <c r="L8" s="4" t="n">
         <v>0.9226</v>
       </c>
-      <c r="M8" s="2" t="n">
+      <c r="M8" s="4" t="n">
         <v>0.8556</v>
       </c>
-      <c r="N8" s="2" t="n">
+      <c r="N8" s="4" t="n">
         <v>0.4476</v>
       </c>
-      <c r="O8" s="2" t="n">
+      <c r="O8" s="4" t="n">
         <v>0.6516999999999999</v>
       </c>
-      <c r="P8" s="2" t="n">
+      <c r="P8" s="4" t="n">
         <v>0.9287</v>
       </c>
-      <c r="Q8" s="2" t="n">
+      <c r="Q8" s="4" t="n">
         <v>0.8854</v>
       </c>
-      <c r="R8" s="2" t="n">
+      <c r="R8" s="4" t="n">
         <v>0.5053</v>
       </c>
-      <c r="S8" s="2" t="n">
+      <c r="S8" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="T8" s="2" t="n">
+      <c r="T8" s="4" t="n">
         <v>0.6463</v>
       </c>
-      <c r="U8" s="2" t="n">
+      <c r="U8" s="4" t="n">
         <v>0.4989</v>
       </c>
       <c r="V8" s="2" t="inlineStr">
@@ -1279,29 +2326,14 @@
           <t>inverted weights</t>
         </is>
       </c>
-      <c r="W8" s="2" t="n">
+      <c r="W8" s="4" t="n">
         <v>-6.31</v>
       </c>
-      <c r="X8" s="2" t="n">
+      <c r="X8" s="4" t="n">
         <v>-10.04</v>
       </c>
-      <c r="Y8" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="Z8" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="AA8" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
+    <row r="9" ht="135" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>conf=0.90 cap=10 seed=0</t>
@@ -1317,7 +2349,7 @@
           <t>pred==gt ∧ conf&gt;0.90</t>
         </is>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" s="4" t="n">
         <v>10</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1325,78 +2357,63 @@
           <t>(1, 1, 0)</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="4" t="n">
         <v>63798</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G9" s="4" t="n">
         <v>0.6403</v>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="4" t="n">
         <v>0.9356</v>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="I9" s="4" t="n">
         <v>0.8639</v>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="J9" s="4" t="n">
         <v>0.4946</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="K9" s="4" t="n">
         <v>0.6996</v>
       </c>
-      <c r="L9" s="2" t="n">
+      <c r="L9" s="4" t="n">
         <v>0.9370000000000001</v>
       </c>
-      <c r="M9" s="2" t="n">
+      <c r="M9" s="4" t="n">
         <v>0.8927</v>
       </c>
-      <c r="N9" s="2" t="n">
+      <c r="N9" s="4" t="n">
         <v>0.5770999999999999</v>
       </c>
-      <c r="O9" s="2" t="n">
+      <c r="O9" s="4" t="n">
         <v>0.7336</v>
       </c>
-      <c r="P9" s="2" t="n">
+      <c r="P9" s="4" t="n">
         <v>0.9373</v>
       </c>
-      <c r="Q9" s="2" t="n">
+      <c r="Q9" s="4" t="n">
         <v>0.9041</v>
       </c>
-      <c r="R9" s="2" t="n">
+      <c r="R9" s="4" t="n">
         <v>0.6264999999999999</v>
       </c>
-      <c r="S9" s="2" t="n">
+      <c r="S9" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="T9" s="2" t="n">
+      <c r="T9" s="4" t="n">
         <v>0.7307</v>
       </c>
-      <c r="U9" s="2" t="n">
+      <c r="U9" s="4" t="n">
         <v>0.6227</v>
       </c>
       <c r="V9" s="2" t="inlineStr"/>
-      <c r="W9" s="2" t="n">
+      <c r="W9" s="4" t="n">
         <v>1.88</v>
       </c>
-      <c r="X9" s="2" t="n">
+      <c r="X9" s="4" t="n">
         <v>2.08</v>
       </c>
-      <c r="Y9" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="Z9" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="AA9" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
+    <row r="10" ht="135" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>conf=0.90 cap=10 seed=1</t>
@@ -1412,7 +2429,7 @@
           <t>pred==gt ∧ conf&gt;0.90</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1420,78 +2437,63 @@
           <t>(1, 1, 0)</t>
         </is>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F10" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="G10" s="4" t="n">
         <v>0.6331</v>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="4" t="n">
         <v>0.9461000000000001</v>
       </c>
-      <c r="I10" s="2" t="n">
+      <c r="I10" s="4" t="n">
         <v>0.8544</v>
       </c>
-      <c r="J10" s="2" t="n">
+      <c r="J10" s="4" t="n">
         <v>0.4852</v>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="K10" s="4" t="n">
         <v>0.6909</v>
       </c>
-      <c r="L10" s="2" t="n">
+      <c r="L10" s="4" t="n">
         <v>0.9487</v>
       </c>
-      <c r="M10" s="2" t="n">
+      <c r="M10" s="4" t="n">
         <v>0.8866000000000001</v>
       </c>
-      <c r="N10" s="2" t="n">
+      <c r="N10" s="4" t="n">
         <v>0.5635</v>
       </c>
-      <c r="O10" s="2" t="n">
+      <c r="O10" s="4" t="n">
         <v>0.725</v>
       </c>
-      <c r="P10" s="2" t="n">
+      <c r="P10" s="4" t="n">
         <v>0.9494</v>
       </c>
-      <c r="Q10" s="2" t="n">
+      <c r="Q10" s="4" t="n">
         <v>0.9021</v>
       </c>
-      <c r="R10" s="2" t="n">
+      <c r="R10" s="4" t="n">
         <v>0.6114000000000001</v>
       </c>
-      <c r="S10" s="2" t="n">
+      <c r="S10" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="T10" s="2" t="n">
+      <c r="T10" s="4" t="n">
         <v>0.725</v>
       </c>
-      <c r="U10" s="2" t="n">
+      <c r="U10" s="4" t="n">
         <v>0.6114000000000001</v>
       </c>
       <c r="V10" s="2" t="inlineStr"/>
-      <c r="W10" s="2" t="n">
+      <c r="W10" s="4" t="n">
         <v>1.02</v>
       </c>
-      <c r="X10" s="2" t="n">
+      <c r="X10" s="4" t="n">
         <v>0.57</v>
       </c>
-      <c r="Y10" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="Z10" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="AA10" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
+    <row r="11" ht="135" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>conf=0.70 cap=10</t>
@@ -1507,7 +2509,7 @@
           <t>pred==gt ∧ conf&gt;0.70</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="4" t="n">
         <v>10</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1515,78 +2517,63 @@
           <t>(1, 1, 0)</t>
         </is>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="F11" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="G11" s="4" t="n">
         <v>0.6453</v>
       </c>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="4" t="n">
         <v>0.9288999999999999</v>
       </c>
-      <c r="I11" s="2" t="n">
+      <c r="I11" s="4" t="n">
         <v>0.8617</v>
       </c>
-      <c r="J11" s="2" t="n">
+      <c r="J11" s="4" t="n">
         <v>0.5047</v>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="K11" s="4" t="n">
         <v>0.698</v>
       </c>
-      <c r="L11" s="2" t="n">
+      <c r="L11" s="4" t="n">
         <v>0.9301</v>
       </c>
-      <c r="M11" s="2" t="n">
+      <c r="M11" s="4" t="n">
         <v>0.886</v>
       </c>
-      <c r="N11" s="2" t="n">
+      <c r="N11" s="4" t="n">
         <v>0.5785</v>
       </c>
-      <c r="O11" s="2" t="n">
+      <c r="O11" s="4" t="n">
         <v>0.7289</v>
       </c>
-      <c r="P11" s="2" t="n">
+      <c r="P11" s="4" t="n">
         <v>0.9304</v>
       </c>
-      <c r="Q11" s="2" t="n">
+      <c r="Q11" s="4" t="n">
         <v>0.8963</v>
       </c>
-      <c r="R11" s="2" t="n">
+      <c r="R11" s="4" t="n">
         <v>0.6234</v>
       </c>
-      <c r="S11" s="2" t="n">
+      <c r="S11" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="T11" s="2" t="n">
+      <c r="T11" s="4" t="n">
         <v>0.7289</v>
       </c>
-      <c r="U11" s="2" t="n">
+      <c r="U11" s="4" t="n">
         <v>0.6234</v>
       </c>
       <c r="V11" s="2" t="inlineStr"/>
-      <c r="W11" s="2" t="n">
+      <c r="W11" s="4" t="n">
         <v>1.41</v>
       </c>
-      <c r="X11" s="2" t="n">
+      <c r="X11" s="4" t="n">
         <v>1.77</v>
       </c>
-      <c r="Y11" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="Z11" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="AA11" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
+    <row r="12" ht="135" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>conf=0.80 cap=10</t>
@@ -1602,7 +2589,7 @@
           <t>pred==gt ∧ conf&gt;0.80</t>
         </is>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D12" s="4" t="n">
         <v>10</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1610,52 +2597,52 @@
           <t>(1, 1, 0)</t>
         </is>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="F12" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="G12" s="4" t="n">
         <v>0.6186</v>
       </c>
-      <c r="H12" s="2" t="n">
+      <c r="H12" s="4" t="n">
         <v>0.9417</v>
       </c>
-      <c r="I12" s="2" t="n">
+      <c r="I12" s="4" t="n">
         <v>0.843</v>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="J12" s="4" t="n">
         <v>0.4675</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="K12" s="4" t="n">
         <v>0.6785</v>
       </c>
-      <c r="L12" s="2" t="n">
+      <c r="L12" s="4" t="n">
         <v>0.9449</v>
       </c>
-      <c r="M12" s="2" t="n">
+      <c r="M12" s="4" t="n">
         <v>0.8769</v>
       </c>
-      <c r="N12" s="2" t="n">
+      <c r="N12" s="4" t="n">
         <v>0.5485</v>
       </c>
-      <c r="O12" s="2" t="n">
+      <c r="O12" s="4" t="n">
         <v>0.7139</v>
       </c>
-      <c r="P12" s="2" t="n">
+      <c r="P12" s="4" t="n">
         <v>0.9455</v>
       </c>
-      <c r="Q12" s="2" t="n">
+      <c r="Q12" s="4" t="n">
         <v>0.8913</v>
       </c>
-      <c r="R12" s="2" t="n">
+      <c r="R12" s="4" t="n">
         <v>0.5988</v>
       </c>
-      <c r="S12" s="2" t="n">
+      <c r="S12" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="T12" s="2" t="n">
+      <c r="T12" s="4" t="n">
         <v>0.7139</v>
       </c>
-      <c r="U12" s="2" t="n">
+      <c r="U12" s="4" t="n">
         <v>0.5988</v>
       </c>
       <c r="V12" s="2" t="inlineStr">
@@ -1663,29 +2650,14 @@
           <t>outlier (lower than expected)</t>
         </is>
       </c>
-      <c r="W12" s="2" t="n">
+      <c r="W12" s="4" t="n">
         <v>-0.09</v>
       </c>
-      <c r="X12" s="2" t="n">
+      <c r="X12" s="4" t="n">
         <v>-0.6899999999999999</v>
       </c>
-      <c r="Y12" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="Z12" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="AA12" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
     </row>
-    <row r="13" ht="22" customHeight="1">
+    <row r="13" ht="135" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>conf=0.95 cap=10</t>
@@ -1701,7 +2673,7 @@
           <t>pred==gt ∧ conf&gt;0.95</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D13" s="4" t="n">
         <v>10</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1709,78 +2681,63 @@
           <t>(1, 1, 0)</t>
         </is>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="F13" s="4" t="n">
         <v>61194</v>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="G13" s="4" t="n">
         <v>0.6453</v>
       </c>
-      <c r="H13" s="2" t="n">
+      <c r="H13" s="4" t="n">
         <v>0.9167</v>
       </c>
-      <c r="I13" s="2" t="n">
+      <c r="I13" s="4" t="n">
         <v>0.8548</v>
       </c>
-      <c r="J13" s="2" t="n">
+      <c r="J13" s="4" t="n">
         <v>0.5098</v>
       </c>
-      <c r="K13" s="2" t="n">
+      <c r="K13" s="4" t="n">
         <v>0.7012</v>
       </c>
-      <c r="L13" s="2" t="n">
+      <c r="L13" s="4" t="n">
         <v>0.9186</v>
       </c>
-      <c r="M13" s="2" t="n">
+      <c r="M13" s="4" t="n">
         <v>0.8837</v>
       </c>
-      <c r="N13" s="2" t="n">
+      <c r="N13" s="4" t="n">
         <v>0.5867</v>
       </c>
-      <c r="O13" s="2" t="n">
+      <c r="O13" s="4" t="n">
         <v>0.733</v>
       </c>
-      <c r="P13" s="2" t="n">
+      <c r="P13" s="4" t="n">
         <v>0.919</v>
       </c>
-      <c r="Q13" s="2" t="n">
+      <c r="Q13" s="4" t="n">
         <v>0.8947000000000001</v>
       </c>
-      <c r="R13" s="2" t="n">
+      <c r="R13" s="4" t="n">
         <v>0.6326000000000001</v>
       </c>
-      <c r="S13" s="2" t="n">
+      <c r="S13" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="T13" s="2" t="n">
+      <c r="T13" s="4" t="n">
         <v>0.7321</v>
       </c>
-      <c r="U13" s="2" t="n">
+      <c r="U13" s="4" t="n">
         <v>0.633</v>
       </c>
       <c r="V13" s="2" t="inlineStr"/>
-      <c r="W13" s="2" t="n">
+      <c r="W13" s="4" t="n">
         <v>1.82</v>
       </c>
-      <c r="X13" s="2" t="n">
+      <c r="X13" s="4" t="n">
         <v>2.69</v>
       </c>
-      <c r="Y13" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="Z13" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="AA13" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
+    <row r="14" ht="135" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>conf=0.99 cap=10</t>
@@ -1796,7 +2753,7 @@
           <t>pred==gt ∧ conf&gt;0.99</t>
         </is>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" s="4" t="n">
         <v>10</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1804,52 +2761,52 @@
           <t>(1, 1, 0)</t>
         </is>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="F14" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="G14" s="4" t="n">
         <v>0.6489</v>
       </c>
-      <c r="H14" s="2" t="n">
+      <c r="H14" s="4" t="n">
         <v>0.9406</v>
       </c>
-      <c r="I14" s="2" t="n">
+      <c r="I14" s="4" t="n">
         <v>0.8611</v>
       </c>
-      <c r="J14" s="2" t="n">
+      <c r="J14" s="4" t="n">
         <v>0.5086000000000001</v>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="K14" s="4" t="n">
         <v>0.7030999999999999</v>
       </c>
-      <c r="L14" s="2" t="n">
+      <c r="L14" s="4" t="n">
         <v>0.9425</v>
       </c>
-      <c r="M14" s="2" t="n">
+      <c r="M14" s="4" t="n">
         <v>0.888</v>
       </c>
-      <c r="N14" s="2" t="n">
+      <c r="N14" s="4" t="n">
         <v>0.5836</v>
       </c>
-      <c r="O14" s="2" t="n">
+      <c r="O14" s="4" t="n">
         <v>0.7355</v>
       </c>
-      <c r="P14" s="2" t="n">
+      <c r="P14" s="4" t="n">
         <v>0.9429999999999999</v>
       </c>
-      <c r="Q14" s="2" t="n">
+      <c r="Q14" s="4" t="n">
         <v>0.9004</v>
       </c>
-      <c r="R14" s="2" t="n">
+      <c r="R14" s="4" t="n">
         <v>0.63</v>
       </c>
-      <c r="S14" s="2" t="n">
+      <c r="S14" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="T14" s="2" t="n">
+      <c r="T14" s="4" t="n">
         <v>0.7355</v>
       </c>
-      <c r="U14" s="2" t="n">
+      <c r="U14" s="4" t="n">
         <v>0.63</v>
       </c>
       <c r="V14" s="2" t="inlineStr">
@@ -1857,29 +2814,14 @@
           <t>stable best</t>
         </is>
       </c>
-      <c r="W14" s="2" t="n">
+      <c r="W14" s="4" t="n">
         <v>2.07</v>
       </c>
-      <c r="X14" s="2" t="n">
+      <c r="X14" s="4" t="n">
         <v>2.43</v>
       </c>
-      <c r="Y14" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="Z14" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="AA14" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
+    <row r="15" ht="135" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>conf=0.99 cap=15</t>
@@ -1895,7 +2837,7 @@
           <t>pred==gt ∧ conf&gt;0.99</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D15" s="4" t="n">
         <v>15</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1903,52 +2845,52 @@
           <t>(1, 1, 0)</t>
         </is>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="F15" s="4" t="n">
         <v>48174</v>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="G15" s="4" t="n">
         <v>0.619</v>
       </c>
-      <c r="H15" s="2" t="n">
+      <c r="H15" s="4" t="n">
         <v>0.9246</v>
       </c>
-      <c r="I15" s="2" t="n">
+      <c r="I15" s="4" t="n">
         <v>0.8367</v>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="J15" s="4" t="n">
         <v>0.474</v>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="K15" s="4" t="n">
         <v>0.6757</v>
       </c>
-      <c r="L15" s="2" t="n">
+      <c r="L15" s="4" t="n">
         <v>0.9283</v>
       </c>
-      <c r="M15" s="2" t="n">
+      <c r="M15" s="4" t="n">
         <v>0.8699</v>
       </c>
-      <c r="N15" s="2" t="n">
+      <c r="N15" s="4" t="n">
         <v>0.5498</v>
       </c>
-      <c r="O15" s="2" t="n">
+      <c r="O15" s="4" t="n">
         <v>0.7077</v>
       </c>
-      <c r="P15" s="2" t="n">
+      <c r="P15" s="4" t="n">
         <v>0.9295</v>
       </c>
-      <c r="Q15" s="2" t="n">
+      <c r="Q15" s="4" t="n">
         <v>0.883</v>
       </c>
-      <c r="R15" s="2" t="n">
+      <c r="R15" s="4" t="n">
         <v>0.5954</v>
       </c>
-      <c r="S15" s="2" t="n">
+      <c r="S15" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="T15" s="2" t="n">
+      <c r="T15" s="4" t="n">
         <v>0.6933</v>
       </c>
-      <c r="U15" s="2" t="n">
+      <c r="U15" s="4" t="n">
         <v>0.581</v>
       </c>
       <c r="V15" s="2" t="inlineStr">
@@ -1956,29 +2898,14 @@
           <t>stable but lower than cap=10</t>
         </is>
       </c>
-      <c r="W15" s="2" t="n">
+      <c r="W15" s="4" t="n">
         <v>-0.71</v>
       </c>
-      <c r="X15" s="2" t="n">
+      <c r="X15" s="4" t="n">
         <v>-1.03</v>
       </c>
-      <c r="Y15" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="Z15" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="AA15" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
+    <row r="16" ht="135" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>conf=0.99 cap=20</t>
@@ -1994,7 +2921,7 @@
           <t>pred==gt ∧ conf&gt;0.99</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D16" s="4" t="n">
         <v>20</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -2002,52 +2929,52 @@
           <t>(1, 1, 0)</t>
         </is>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F16" s="4" t="n">
         <v>39060</v>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="G16" s="4" t="n">
         <v>0.6481</v>
       </c>
-      <c r="H16" s="2" t="n">
+      <c r="H16" s="4" t="n">
         <v>0.9330000000000001</v>
       </c>
-      <c r="I16" s="2" t="n">
+      <c r="I16" s="4" t="n">
         <v>0.8588</v>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="J16" s="4" t="n">
         <v>0.5097</v>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="K16" s="4" t="n">
         <v>0.7074</v>
       </c>
-      <c r="L16" s="2" t="n">
+      <c r="L16" s="4" t="n">
         <v>0.9351</v>
       </c>
-      <c r="M16" s="2" t="n">
+      <c r="M16" s="4" t="n">
         <v>0.8895999999999999</v>
       </c>
-      <c r="N16" s="2" t="n">
+      <c r="N16" s="4" t="n">
         <v>0.5911</v>
       </c>
-      <c r="O16" s="2" t="n">
+      <c r="O16" s="4" t="n">
         <v>0.7431</v>
       </c>
-      <c r="P16" s="2" t="n">
+      <c r="P16" s="4" t="n">
         <v>0.9355</v>
       </c>
-      <c r="Q16" s="2" t="n">
+      <c r="Q16" s="4" t="n">
         <v>0.9032</v>
       </c>
-      <c r="R16" s="2" t="n">
+      <c r="R16" s="4" t="n">
         <v>0.6423</v>
       </c>
-      <c r="S16" s="2" t="n">
+      <c r="S16" s="4" t="n">
         <v>65100</v>
       </c>
-      <c r="T16" s="2" t="n">
+      <c r="T16" s="4" t="n">
         <v>0.0176</v>
       </c>
-      <c r="U16" s="2" t="n">
+      <c r="U16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V16" s="2" t="inlineStr">
@@ -2055,26 +2982,11 @@
           <t>peak 0.7431 then collapses to 0.0176</t>
         </is>
       </c>
-      <c r="W16" s="2" t="n">
+      <c r="W16" s="4" t="n">
         <v>2.83</v>
       </c>
-      <c r="X16" s="2" t="n">
+      <c r="X16" s="4" t="n">
         <v>3.66</v>
-      </c>
-      <c r="Y16" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="Z16" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
-      </c>
-      <c r="AA16" s="3" t="inlineStr">
-        <is>
-          <t>📊 View</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -2176,66 +3088,22 @@
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA2" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z3" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA3" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y4" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z4" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA4" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y5" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z5" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA5" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y6" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z6" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA6" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y7" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z7" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA7" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y8" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z8" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA8" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y9" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z9" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA9" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y10" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z10" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA10" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y11" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z11" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA11" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y12" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z12" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA12" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y13" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z13" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA13" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y14" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z14" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA14" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y15" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z15" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA15" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y16" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z16" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA16" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
xlsx: embed images at full resolution (1089x645) for clarity; file 2.87 MB
</commit_message>
<xml_diff>
--- a/on-the-fly-supervision.xlsx
+++ b/on-the-fly-supervision.xlsx
@@ -176,7 +176,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -201,7 +201,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -226,7 +226,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -251,7 +251,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10344150" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -276,7 +276,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10344150" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="5" name="Image 5" descr="Picture"/>
@@ -301,7 +301,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10344150" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="6" name="Image 6" descr="Picture"/>
@@ -326,7 +326,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="7" name="Image 7" descr="Picture"/>
@@ -351,7 +351,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="8" name="Image 8" descr="Picture"/>
@@ -376,7 +376,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -401,7 +401,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2619375" cy="1619250"/>
+    <ext cx="9772650" cy="6038850"/>
     <pic>
       <nvPicPr>
         <cNvPr id="10" name="Image 10" descr="Picture"/>
@@ -426,7 +426,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2619375" cy="1619250"/>
+    <ext cx="9772650" cy="6038850"/>
     <pic>
       <nvPicPr>
         <cNvPr id="11" name="Image 11" descr="Picture"/>
@@ -451,7 +451,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2619375" cy="1619250"/>
+    <ext cx="9772650" cy="6038850"/>
     <pic>
       <nvPicPr>
         <cNvPr id="12" name="Image 12" descr="Picture"/>
@@ -476,7 +476,7 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="13" name="Image 13" descr="Picture"/>
@@ -501,7 +501,7 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="14" name="Image 14" descr="Picture"/>
@@ -526,7 +526,7 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="15" name="Image 15" descr="Picture"/>
@@ -551,7 +551,7 @@
       <row>6</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="16" name="Image 16" descr="Picture"/>
@@ -576,7 +576,7 @@
       <row>6</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="17" name="Image 17" descr="Picture"/>
@@ -601,7 +601,7 @@
       <row>6</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="18" name="Image 18" descr="Picture"/>
@@ -626,7 +626,7 @@
       <row>7</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="19" name="Image 19" descr="Picture"/>
@@ -651,7 +651,7 @@
       <row>7</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="20" name="Image 20" descr="Picture"/>
@@ -676,7 +676,7 @@
       <row>7</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="21" name="Image 21" descr="Picture"/>
@@ -701,7 +701,7 @@
       <row>8</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="22" name="Image 22" descr="Picture"/>
@@ -726,7 +726,7 @@
       <row>8</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="23" name="Image 23" descr="Picture"/>
@@ -751,7 +751,7 @@
       <row>8</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="24" name="Image 24" descr="Picture"/>
@@ -776,7 +776,7 @@
       <row>9</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="25" name="Image 25" descr="Picture"/>
@@ -801,7 +801,7 @@
       <row>9</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="26" name="Image 26" descr="Picture"/>
@@ -826,7 +826,7 @@
       <row>9</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="27" name="Image 27" descr="Picture"/>
@@ -851,7 +851,7 @@
       <row>10</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="28" name="Image 28" descr="Picture"/>
@@ -876,7 +876,7 @@
       <row>10</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="29" name="Image 29" descr="Picture"/>
@@ -901,7 +901,7 @@
       <row>10</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="30" name="Image 30" descr="Picture"/>
@@ -926,7 +926,7 @@
       <row>11</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="31" name="Image 31" descr="Picture"/>
@@ -951,7 +951,7 @@
       <row>11</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="32" name="Image 32" descr="Picture"/>
@@ -976,7 +976,7 @@
       <row>11</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="33" name="Image 33" descr="Picture"/>
@@ -1001,7 +1001,7 @@
       <row>12</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="34" name="Image 34" descr="Picture"/>
@@ -1026,7 +1026,7 @@
       <row>12</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="35" name="Image 35" descr="Picture"/>
@@ -1051,7 +1051,7 @@
       <row>12</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="36" name="Image 36" descr="Picture"/>
@@ -1076,7 +1076,7 @@
       <row>13</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="37" name="Image 37" descr="Picture"/>
@@ -1101,7 +1101,7 @@
       <row>13</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="38" name="Image 38" descr="Picture"/>
@@ -1126,7 +1126,7 @@
       <row>13</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="39" name="Image 39" descr="Picture"/>
@@ -1151,7 +1151,7 @@
       <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="40" name="Image 40" descr="Picture"/>
@@ -1176,7 +1176,7 @@
       <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="41" name="Image 41" descr="Picture"/>
@@ -1201,7 +1201,7 @@
       <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="42" name="Image 42" descr="Picture"/>
@@ -1226,7 +1226,7 @@
       <row>15</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="43" name="Image 43" descr="Picture"/>
@@ -1251,7 +1251,7 @@
       <row>15</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="44" name="Image 44" descr="Picture"/>
@@ -1276,7 +1276,7 @@
       <row>15</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2667000" cy="1581150"/>
+    <ext cx="10372725" cy="6143625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="45" name="Image 45" descr="Picture"/>
@@ -1613,9 +1613,9 @@
     <col width="26" customWidth="1" min="22" max="22"/>
     <col width="11" customWidth="1" min="23" max="23"/>
     <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="40" customWidth="1" min="25" max="25"/>
-    <col width="40" customWidth="1" min="26" max="26"/>
-    <col width="40" customWidth="1" min="27" max="27"/>
+    <col width="215" customWidth="1" min="25" max="25"/>
+    <col width="215" customWidth="1" min="26" max="26"/>
+    <col width="215" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1755,7 +1755,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="135" customHeight="1">
+    <row r="2" ht="675" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>baseline</t>
@@ -1841,7 +1841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" ht="135" customHeight="1">
+    <row r="3" ht="675" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>v2 (cap=∞, no filter)</t>
@@ -1927,7 +1927,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="4" ht="135" customHeight="1">
+    <row r="4" ht="675" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>c20 (cap=20, no filter)</t>
@@ -2007,7 +2007,7 @@
         <v>-4.27</v>
       </c>
     </row>
-    <row r="5" ht="135" customHeight="1">
+    <row r="5" ht="675" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>M3 (cap=10, no filter)</t>
@@ -2087,7 +2087,7 @@
         <v>-8.050000000000001</v>
       </c>
     </row>
-    <row r="6" ht="135" customHeight="1">
+    <row r="6" ht="675" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>c5 (cap=5, no filter)</t>
@@ -2167,7 +2167,7 @@
         <v>-31.5</v>
       </c>
     </row>
-    <row r="7" ht="135" customHeight="1">
+    <row r="7" ht="675" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>M2 (clue only)</t>
@@ -2249,7 +2249,7 @@
         <v>-51.33</v>
       </c>
     </row>
-    <row r="8" ht="135" customHeight="1">
+    <row r="8" ht="675" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>inverse_mask cap=10</t>
@@ -2333,7 +2333,7 @@
         <v>-10.04</v>
       </c>
     </row>
-    <row r="9" ht="135" customHeight="1">
+    <row r="9" ht="675" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>conf=0.90 cap=10 seed=0</t>
@@ -2413,7 +2413,7 @@
         <v>2.08</v>
       </c>
     </row>
-    <row r="10" ht="135" customHeight="1">
+    <row r="10" ht="675" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>conf=0.90 cap=10 seed=1</t>
@@ -2493,7 +2493,7 @@
         <v>0.57</v>
       </c>
     </row>
-    <row r="11" ht="135" customHeight="1">
+    <row r="11" ht="675" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>conf=0.70 cap=10</t>
@@ -2573,7 +2573,7 @@
         <v>1.77</v>
       </c>
     </row>
-    <row r="12" ht="135" customHeight="1">
+    <row r="12" ht="675" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>conf=0.80 cap=10</t>
@@ -2657,7 +2657,7 @@
         <v>-0.6899999999999999</v>
       </c>
     </row>
-    <row r="13" ht="135" customHeight="1">
+    <row r="13" ht="675" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>conf=0.95 cap=10</t>
@@ -2737,7 +2737,7 @@
         <v>2.69</v>
       </c>
     </row>
-    <row r="14" ht="135" customHeight="1">
+    <row r="14" ht="675" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>conf=0.99 cap=10</t>
@@ -2821,7 +2821,7 @@
         <v>2.43</v>
       </c>
     </row>
-    <row r="15" ht="135" customHeight="1">
+    <row r="15" ht="675" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>conf=0.99 cap=15</t>
@@ -2905,7 +2905,7 @@
         <v>-1.03</v>
       </c>
     </row>
-    <row r="16" ht="135" customHeight="1">
+    <row r="16" ht="675" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>conf=0.99 cap=20</t>

</xml_diff>